<commit_message>
Add Current group active/passive state to Current group Excel template
</commit_message>
<xml_diff>
--- a/wwwroot/templates/CariGrupTemplate.xlsx
+++ b/wwwroot/templates/CariGrupTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOD\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0471D824-BD7E-4113-BABA-2C3D6F11A0FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{551906FB-949D-4D26-AF9A-FA3934F53DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2460" yWindow="2175" windowWidth="18825" windowHeight="11130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="18795" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>CariGrupAdi</t>
   </si>
   <si>
     <t>CariGrupId</t>
+  </si>
+  <si>
+    <t>CariGrupAktifPasif</t>
   </si>
 </sst>
 </file>
@@ -365,19 +368,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Change excel templates with filled ones for testing
</commit_message>
<xml_diff>
--- a/wwwroot/templates/CariGrupTemplate.xlsx
+++ b/wwwroot/templates/CariGrupTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMutabakat\wwwroot\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOD\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{551906FB-949D-4D26-AF9A-FA3934F53DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9978F6A2-C409-49DC-993C-A34FF3D6884B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="18795" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7185" yWindow="6210" windowWidth="16950" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>CariGrupAdi</t>
   </si>
@@ -29,6 +29,18 @@
   </si>
   <si>
     <t>CariGrupAktifPasif</t>
+  </si>
+  <si>
+    <t>Müşteriler</t>
+  </si>
+  <si>
+    <t>Tedarikçiler</t>
+  </si>
+  <si>
+    <t>Bayiler</t>
+  </si>
+  <si>
+    <t>Eski Cariler</t>
   </si>
 </sst>
 </file>
@@ -368,12 +380,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -385,6 +395,50 @@
       </c>
       <c r="C1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>